<commit_message>
updated the production logger
</commit_message>
<xml_diff>
--- a/data/GARMENT_ORDERPRODUCTION_DETAILS.xlsx
+++ b/data/GARMENT_ORDERPRODUCTION_DETAILS.xlsx
@@ -1,10 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="4" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\head user\Desktop\Hamthan\Clinets\2-Factor\Backend\data\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="120" yWindow="105" windowWidth="28695" windowHeight="12540" firstSheet="7" activeTab="12"/>
+    <workbookView minimized="1" xWindow="120" yWindow="105" windowWidth="28695" windowHeight="12540" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="KJ GARMENT ORDER" sheetId="3" r:id="rId1"/>
@@ -21,7 +26,7 @@
     <sheet name="NIPAL-NEW GARMENT ORDER" sheetId="12" r:id="rId12"/>
     <sheet name="NIPAL-NEW PRODUCTION" sheetId="13" r:id="rId13"/>
   </sheets>
-  <calcPr calcId="145621"/>
+  <calcPr calcId="152511"/>
 </workbook>
 </file>
 
@@ -1192,6 +1197,12 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1219,19 +1230,13 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1240,20 +1245,11 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1265,6 +1261,15 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1309,6 +1314,12 @@
     <xf numFmtId="0" fontId="10" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="20" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1321,12 +1332,6 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1336,6 +1341,9 @@
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -1384,7 +1392,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -1419,7 +1427,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -1640,22 +1648,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="27" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="83" t="s">
+      <c r="A1" s="85" t="s">
         <v>31</v>
       </c>
-      <c r="B1" s="84"/>
-      <c r="C1" s="84"/>
-      <c r="D1" s="84"/>
-      <c r="E1" s="84"/>
-      <c r="F1" s="84"/>
-      <c r="G1" s="84"/>
-      <c r="H1" s="84"/>
-      <c r="I1" s="84"/>
-      <c r="J1" s="84"/>
-      <c r="K1" s="84"/>
-      <c r="L1" s="84"/>
-      <c r="M1" s="84"/>
-      <c r="N1" s="85"/>
+      <c r="B1" s="86"/>
+      <c r="C1" s="86"/>
+      <c r="D1" s="86"/>
+      <c r="E1" s="86"/>
+      <c r="F1" s="86"/>
+      <c r="G1" s="86"/>
+      <c r="H1" s="86"/>
+      <c r="I1" s="86"/>
+      <c r="J1" s="86"/>
+      <c r="K1" s="86"/>
+      <c r="L1" s="86"/>
+      <c r="M1" s="86"/>
+      <c r="N1" s="87"/>
     </row>
     <row r="2" spans="1:18" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
@@ -1693,7 +1701,7 @@
       <c r="A3" s="4">
         <v>1</v>
       </c>
-      <c r="B3" s="86" t="s">
+      <c r="B3" s="88" t="s">
         <v>33</v>
       </c>
       <c r="C3" s="5" t="s">
@@ -1726,7 +1734,7 @@
       <c r="A4" s="4">
         <v>2</v>
       </c>
-      <c r="B4" s="87"/>
+      <c r="B4" s="89"/>
       <c r="C4" s="5" t="s">
         <v>35</v>
       </c>
@@ -1819,7 +1827,7 @@
       <c r="A10" s="4">
         <v>3</v>
       </c>
-      <c r="B10" s="86" t="s">
+      <c r="B10" s="88" t="s">
         <v>36</v>
       </c>
       <c r="C10" s="5" t="s">
@@ -1864,7 +1872,7 @@
       <c r="A11" s="4">
         <v>4</v>
       </c>
-      <c r="B11" s="88"/>
+      <c r="B11" s="90"/>
       <c r="C11" s="5" t="s">
         <v>35</v>
       </c>
@@ -1907,7 +1915,7 @@
       <c r="A12" s="4">
         <v>5</v>
       </c>
-      <c r="B12" s="87"/>
+      <c r="B12" s="89"/>
       <c r="C12" s="5" t="s">
         <v>37</v>
       </c>
@@ -2023,7 +2031,7 @@
       <c r="A18" s="4">
         <v>1</v>
       </c>
-      <c r="B18" s="89" t="s">
+      <c r="B18" s="91" t="s">
         <v>38</v>
       </c>
       <c r="C18" s="5" t="s">
@@ -2077,7 +2085,7 @@
       <c r="A19" s="4">
         <v>2</v>
       </c>
-      <c r="B19" s="90"/>
+      <c r="B19" s="92"/>
       <c r="C19" s="5" t="s">
         <v>35</v>
       </c>
@@ -2129,7 +2137,7 @@
       <c r="A20" s="4">
         <v>3</v>
       </c>
-      <c r="B20" s="91"/>
+      <c r="B20" s="93"/>
       <c r="C20" s="5" t="s">
         <v>37</v>
       </c>
@@ -2222,7 +2230,7 @@
       <c r="A26" s="4">
         <v>1</v>
       </c>
-      <c r="B26" s="89" t="s">
+      <c r="B26" s="91" t="s">
         <v>40</v>
       </c>
       <c r="C26" s="5" t="s">
@@ -2258,7 +2266,7 @@
       <c r="A27" s="4">
         <v>2</v>
       </c>
-      <c r="B27" s="90"/>
+      <c r="B27" s="92"/>
       <c r="C27" s="5" t="s">
         <v>35</v>
       </c>
@@ -2292,7 +2300,7 @@
       <c r="A28" s="4">
         <v>3</v>
       </c>
-      <c r="B28" s="91"/>
+      <c r="B28" s="93"/>
       <c r="C28" s="5" t="s">
         <v>37</v>
       </c>
@@ -2347,11 +2355,11 @@
     </row>
     <row r="34" spans="7:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="35" spans="7:10" ht="29.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="G35" s="92" t="s">
+      <c r="G35" s="83" t="s">
         <v>8</v>
       </c>
-      <c r="H35" s="93"/>
-      <c r="I35" s="93"/>
+      <c r="H35" s="84"/>
+      <c r="I35" s="84"/>
       <c r="J35" s="42">
         <f>J6+N14+Q22+K30</f>
         <v>347</v>
@@ -5049,7 +5057,7 @@
       </c>
     </row>
     <row r="3" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="105" t="s">
+      <c r="A3" s="102" t="s">
         <v>135</v>
       </c>
       <c r="B3" s="59" t="s">
@@ -5078,7 +5086,7 @@
       </c>
     </row>
     <row r="4" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="106"/>
+      <c r="A4" s="103"/>
       <c r="B4" s="59" t="s">
         <v>87</v>
       </c>
@@ -5105,7 +5113,7 @@
       </c>
     </row>
     <row r="5" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="106"/>
+      <c r="A5" s="103"/>
       <c r="B5" s="59" t="s">
         <v>137</v>
       </c>
@@ -5132,7 +5140,7 @@
       </c>
     </row>
     <row r="6" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="106"/>
+      <c r="A6" s="103"/>
       <c r="B6" s="59" t="s">
         <v>138</v>
       </c>
@@ -5159,7 +5167,7 @@
       </c>
     </row>
     <row r="7" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="106"/>
+      <c r="A7" s="103"/>
       <c r="B7" s="59" t="s">
         <v>139</v>
       </c>
@@ -5186,7 +5194,7 @@
       </c>
     </row>
     <row r="8" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="106"/>
+      <c r="A8" s="103"/>
       <c r="B8" s="59" t="s">
         <v>140</v>
       </c>
@@ -5213,7 +5221,7 @@
       </c>
     </row>
     <row r="9" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="106"/>
+      <c r="A9" s="103"/>
       <c r="B9" s="59" t="s">
         <v>141</v>
       </c>
@@ -5240,7 +5248,7 @@
       </c>
     </row>
     <row r="10" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="107"/>
+      <c r="A10" s="104"/>
       <c r="B10" s="59" t="s">
         <v>142</v>
       </c>
@@ -5518,7 +5526,7 @@
       </c>
     </row>
     <row r="35" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="105" t="s">
+      <c r="A35" s="102" t="s">
         <v>135</v>
       </c>
       <c r="B35" s="59" t="s">
@@ -5550,7 +5558,7 @@
       </c>
     </row>
     <row r="36" spans="1:11" s="20" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="106"/>
+      <c r="A36" s="103"/>
       <c r="B36" s="18" t="s">
         <v>141</v>
       </c>
@@ -5580,7 +5588,7 @@
       </c>
     </row>
     <row r="37" spans="1:11" s="20" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="106"/>
+      <c r="A37" s="103"/>
       <c r="B37" s="18" t="s">
         <v>142</v>
       </c>
@@ -5610,7 +5618,7 @@
       </c>
     </row>
     <row r="38" spans="1:11" s="20" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="107"/>
+      <c r="A38" s="104"/>
       <c r="B38" s="18" t="s">
         <v>145</v>
       </c>
@@ -5911,7 +5919,7 @@
       </c>
     </row>
     <row r="65" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A65" s="94" t="s">
+      <c r="A65" s="100" t="s">
         <v>135</v>
       </c>
       <c r="B65" s="59" t="s">
@@ -5943,7 +5951,7 @@
       </c>
     </row>
     <row r="66" spans="1:11" s="20" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A66" s="94"/>
+      <c r="A66" s="100"/>
       <c r="B66" s="18" t="s">
         <v>139</v>
       </c>
@@ -5973,7 +5981,7 @@
       </c>
     </row>
     <row r="67" spans="1:11" s="20" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A67" s="94"/>
+      <c r="A67" s="100"/>
       <c r="B67" s="59" t="s">
         <v>140</v>
       </c>
@@ -6003,7 +6011,7 @@
       </c>
     </row>
     <row r="68" spans="1:11" s="20" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A68" s="94"/>
+      <c r="A68" s="100"/>
       <c r="B68" s="18" t="s">
         <v>141</v>
       </c>
@@ -6034,7 +6042,7 @@
       </c>
     </row>
     <row r="69" spans="1:11" s="20" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A69" s="94"/>
+      <c r="A69" s="100"/>
       <c r="B69" s="18" t="s">
         <v>142</v>
       </c>
@@ -6333,7 +6341,7 @@
       </c>
     </row>
     <row r="96" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A96" s="105" t="s">
+      <c r="A96" s="102" t="s">
         <v>135</v>
       </c>
       <c r="B96" s="59" t="s">
@@ -6365,7 +6373,7 @@
       </c>
     </row>
     <row r="97" spans="1:11" s="20" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A97" s="106"/>
+      <c r="A97" s="103"/>
       <c r="B97" s="18" t="s">
         <v>141</v>
       </c>
@@ -6395,7 +6403,7 @@
       </c>
     </row>
     <row r="98" spans="1:11" s="20" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A98" s="107"/>
+      <c r="A98" s="104"/>
       <c r="B98" s="18"/>
       <c r="C98" s="50">
         <v>0</v>
@@ -6690,7 +6698,7 @@
       </c>
     </row>
     <row r="122" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A122" s="105" t="s">
+      <c r="A122" s="102" t="s">
         <v>135</v>
       </c>
       <c r="B122" s="59" t="s">
@@ -6722,7 +6730,7 @@
       </c>
     </row>
     <row r="123" spans="1:11" s="20" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A123" s="106"/>
+      <c r="A123" s="103"/>
       <c r="B123" s="18" t="s">
         <v>141</v>
       </c>
@@ -6752,7 +6760,7 @@
       </c>
     </row>
     <row r="124" spans="1:11" s="20" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A124" s="107"/>
+      <c r="A124" s="104"/>
       <c r="B124" s="18"/>
       <c r="C124" s="49">
         <v>0</v>
@@ -7049,7 +7057,7 @@
       </c>
     </row>
     <row r="151" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A151" s="105" t="s">
+      <c r="A151" s="102" t="s">
         <v>135</v>
       </c>
       <c r="B151" s="18" t="s">
@@ -7081,7 +7089,7 @@
       </c>
     </row>
     <row r="152" spans="1:11" s="20" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A152" s="106"/>
+      <c r="A152" s="103"/>
       <c r="B152" s="18" t="s">
         <v>142</v>
       </c>
@@ -7111,7 +7119,7 @@
       </c>
     </row>
     <row r="153" spans="1:11" s="20" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A153" s="107"/>
+      <c r="A153" s="104"/>
       <c r="B153" s="18" t="s">
         <v>145</v>
       </c>
@@ -7395,22 +7403,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="27" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="83" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="84"/>
-      <c r="C1" s="84"/>
-      <c r="D1" s="84"/>
-      <c r="E1" s="84"/>
-      <c r="F1" s="84"/>
-      <c r="G1" s="84"/>
-      <c r="H1" s="84"/>
-      <c r="I1" s="84"/>
-      <c r="J1" s="84"/>
-      <c r="K1" s="84"/>
-      <c r="L1" s="84"/>
-      <c r="M1" s="84"/>
-      <c r="N1" s="85"/>
+      <c r="A1" s="85" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="86"/>
+      <c r="C1" s="86"/>
+      <c r="D1" s="86"/>
+      <c r="E1" s="86"/>
+      <c r="F1" s="86"/>
+      <c r="G1" s="86"/>
+      <c r="H1" s="86"/>
+      <c r="I1" s="86"/>
+      <c r="J1" s="86"/>
+      <c r="K1" s="86"/>
+      <c r="L1" s="86"/>
+      <c r="M1" s="86"/>
+      <c r="N1" s="87"/>
     </row>
     <row r="2" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
@@ -7885,18 +7893,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="36.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.65">
-      <c r="A1" s="122" t="s">
+      <c r="A1" s="124" t="s">
         <v>156</v>
       </c>
-      <c r="B1" s="123"/>
-      <c r="C1" s="123"/>
-      <c r="D1" s="123"/>
-      <c r="E1" s="123"/>
-      <c r="F1" s="123"/>
-      <c r="G1" s="123"/>
-      <c r="H1" s="123"/>
-      <c r="I1" s="123"/>
-      <c r="J1" s="124"/>
+      <c r="B1" s="125"/>
+      <c r="C1" s="125"/>
+      <c r="D1" s="125"/>
+      <c r="E1" s="125"/>
+      <c r="F1" s="125"/>
+      <c r="G1" s="125"/>
+      <c r="H1" s="125"/>
+      <c r="I1" s="125"/>
+      <c r="J1" s="126"/>
     </row>
     <row r="2" spans="1:11" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="119" t="s">
@@ -7943,7 +7951,7 @@
       </c>
     </row>
     <row r="4" spans="1:11" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="125"/>
+      <c r="A4" s="127"/>
       <c r="B4" s="81" t="s">
         <v>141</v>
       </c>
@@ -7973,7 +7981,7 @@
       </c>
     </row>
     <row r="5" spans="1:11" s="20" customFormat="1" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="126"/>
+      <c r="A5" s="122"/>
       <c r="B5" s="82" t="s">
         <v>142</v>
       </c>
@@ -8003,7 +8011,7 @@
       </c>
     </row>
     <row r="6" spans="1:11" s="20" customFormat="1" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="126"/>
+      <c r="A6" s="122"/>
       <c r="B6" s="82" t="s">
         <v>145</v>
       </c>
@@ -8258,18 +8266,18 @@
     </row>
     <row r="30" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="31" spans="1:11" ht="36.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.65">
-      <c r="A31" s="122" t="s">
+      <c r="A31" s="124" t="s">
         <v>156</v>
       </c>
-      <c r="B31" s="123"/>
-      <c r="C31" s="123"/>
-      <c r="D31" s="123"/>
-      <c r="E31" s="123"/>
-      <c r="F31" s="123"/>
-      <c r="G31" s="123"/>
-      <c r="H31" s="123"/>
-      <c r="I31" s="123"/>
-      <c r="J31" s="124"/>
+      <c r="B31" s="125"/>
+      <c r="C31" s="125"/>
+      <c r="D31" s="125"/>
+      <c r="E31" s="125"/>
+      <c r="F31" s="125"/>
+      <c r="G31" s="125"/>
+      <c r="H31" s="125"/>
+      <c r="I31" s="125"/>
+      <c r="J31" s="126"/>
     </row>
     <row r="32" spans="1:11" ht="29.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A32" s="119" t="s">
@@ -8316,7 +8324,7 @@
       </c>
     </row>
     <row r="34" spans="1:11" s="20" customFormat="1" ht="45.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="126"/>
+      <c r="A34" s="122"/>
       <c r="B34" s="82" t="s">
         <v>145</v>
       </c>
@@ -8346,7 +8354,7 @@
       </c>
     </row>
     <row r="35" spans="1:11" s="20" customFormat="1" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="126"/>
+      <c r="A35" s="122"/>
       <c r="B35" s="82"/>
       <c r="C35" s="19"/>
       <c r="D35" s="19"/>
@@ -8358,7 +8366,7 @@
       <c r="J35" s="19"/>
     </row>
     <row r="36" spans="1:11" s="20" customFormat="1" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="127"/>
+      <c r="A36" s="123"/>
       <c r="B36" s="82"/>
       <c r="C36" s="19"/>
       <c r="D36" s="19"/>
@@ -8622,18 +8630,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="28.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="101" t="s">
+      <c r="A1" s="94" t="s">
         <v>41</v>
       </c>
-      <c r="B1" s="102"/>
-      <c r="C1" s="96"/>
-      <c r="D1" s="96"/>
-      <c r="E1" s="96"/>
-      <c r="F1" s="96"/>
-      <c r="G1" s="96"/>
-      <c r="H1" s="96"/>
-      <c r="I1" s="96"/>
-      <c r="J1" s="103"/>
+      <c r="B1" s="99"/>
+      <c r="C1" s="95"/>
+      <c r="D1" s="95"/>
+      <c r="E1" s="95"/>
+      <c r="F1" s="95"/>
+      <c r="G1" s="95"/>
+      <c r="H1" s="95"/>
+      <c r="I1" s="95"/>
+      <c r="J1" s="96"/>
       <c r="K1" s="43" t="s">
         <v>42</v>
       </c>
@@ -8642,7 +8650,7 @@
       <c r="N1" s="45"/>
     </row>
     <row r="2" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="94" t="s">
+      <c r="A2" s="100" t="s">
         <v>43</v>
       </c>
       <c r="B2" s="40" t="s">
@@ -8674,7 +8682,7 @@
       </c>
     </row>
     <row r="3" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="94"/>
+      <c r="A3" s="100"/>
       <c r="B3" s="48" t="s">
         <v>45</v>
       </c>
@@ -8704,7 +8712,7 @@
       </c>
     </row>
     <row r="4" spans="1:14" s="20" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="94"/>
+      <c r="A4" s="100"/>
       <c r="B4" s="48" t="s">
         <v>46</v>
       </c>
@@ -8734,7 +8742,7 @@
       </c>
     </row>
     <row r="5" spans="1:14" s="20" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="94"/>
+      <c r="A5" s="100"/>
       <c r="B5" s="18" t="s">
         <v>47</v>
       </c>
@@ -8764,7 +8772,7 @@
       </c>
     </row>
     <row r="6" spans="1:14" s="20" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="94"/>
+      <c r="A6" s="100"/>
       <c r="B6" s="18" t="s">
         <v>48</v>
       </c>
@@ -8794,7 +8802,7 @@
       </c>
     </row>
     <row r="7" spans="1:14" s="20" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="94"/>
+      <c r="A7" s="100"/>
       <c r="B7" s="18" t="s">
         <v>49</v>
       </c>
@@ -8824,7 +8832,7 @@
       </c>
     </row>
     <row r="8" spans="1:14" s="20" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="94"/>
+      <c r="A8" s="100"/>
       <c r="B8" s="18" t="s">
         <v>50</v>
       </c>
@@ -9075,25 +9083,25 @@
     </row>
     <row r="29" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="30" spans="1:14" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="101" t="s">
+      <c r="A30" s="94" t="s">
         <v>52</v>
       </c>
-      <c r="B30" s="102"/>
-      <c r="C30" s="102"/>
-      <c r="D30" s="102"/>
-      <c r="E30" s="102"/>
-      <c r="F30" s="102"/>
-      <c r="G30" s="102"/>
-      <c r="H30" s="102"/>
-      <c r="I30" s="102"/>
-      <c r="J30" s="104"/>
+      <c r="B30" s="99"/>
+      <c r="C30" s="99"/>
+      <c r="D30" s="99"/>
+      <c r="E30" s="99"/>
+      <c r="F30" s="99"/>
+      <c r="G30" s="99"/>
+      <c r="H30" s="99"/>
+      <c r="I30" s="99"/>
+      <c r="J30" s="101"/>
       <c r="K30" s="97"/>
       <c r="L30" s="98"/>
       <c r="M30" s="45"/>
       <c r="N30" s="45"/>
     </row>
     <row r="31" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="105" t="s">
+      <c r="A31" s="102" t="s">
         <v>43</v>
       </c>
       <c r="B31" s="40" t="s">
@@ -9125,7 +9133,7 @@
       </c>
     </row>
     <row r="32" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="106"/>
+      <c r="A32" s="103"/>
       <c r="B32" s="59" t="s">
         <v>53</v>
       </c>
@@ -9155,7 +9163,7 @@
       </c>
     </row>
     <row r="33" spans="1:11" s="20" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="106"/>
+      <c r="A33" s="103"/>
       <c r="B33" s="18" t="s">
         <v>54</v>
       </c>
@@ -9185,7 +9193,7 @@
       </c>
     </row>
     <row r="34" spans="1:11" s="20" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="106"/>
+      <c r="A34" s="103"/>
       <c r="B34" s="18" t="s">
         <v>55</v>
       </c>
@@ -9215,7 +9223,7 @@
       </c>
     </row>
     <row r="35" spans="1:11" s="20" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="106"/>
+      <c r="A35" s="103"/>
       <c r="B35" s="48" t="s">
         <v>45</v>
       </c>
@@ -9245,7 +9253,7 @@
       </c>
     </row>
     <row r="36" spans="1:11" s="20" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="106"/>
+      <c r="A36" s="103"/>
       <c r="B36" s="48" t="s">
         <v>46</v>
       </c>
@@ -9276,7 +9284,7 @@
       </c>
     </row>
     <row r="37" spans="1:11" s="20" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="106"/>
+      <c r="A37" s="103"/>
       <c r="B37" s="18" t="s">
         <v>47</v>
       </c>
@@ -9306,7 +9314,7 @@
       </c>
     </row>
     <row r="38" spans="1:11" s="20" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="106"/>
+      <c r="A38" s="103"/>
       <c r="B38" s="18" t="s">
         <v>56</v>
       </c>
@@ -9336,7 +9344,7 @@
       </c>
     </row>
     <row r="39" spans="1:11" s="20" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="107"/>
+      <c r="A39" s="104"/>
       <c r="B39" s="18" t="s">
         <v>57</v>
       </c>
@@ -9592,25 +9600,25 @@
     </row>
     <row r="60" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="61" spans="1:14" ht="28.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A61" s="101" t="s">
+      <c r="A61" s="94" t="s">
         <v>59</v>
       </c>
-      <c r="B61" s="96"/>
-      <c r="C61" s="96"/>
-      <c r="D61" s="96"/>
-      <c r="E61" s="96"/>
-      <c r="F61" s="96"/>
-      <c r="G61" s="96"/>
-      <c r="H61" s="96"/>
-      <c r="I61" s="96"/>
-      <c r="J61" s="103"/>
+      <c r="B61" s="95"/>
+      <c r="C61" s="95"/>
+      <c r="D61" s="95"/>
+      <c r="E61" s="95"/>
+      <c r="F61" s="95"/>
+      <c r="G61" s="95"/>
+      <c r="H61" s="95"/>
+      <c r="I61" s="95"/>
+      <c r="J61" s="96"/>
       <c r="K61" s="97"/>
       <c r="L61" s="98"/>
       <c r="M61" s="45"/>
       <c r="N61" s="45"/>
     </row>
     <row r="62" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A62" s="94" t="s">
+      <c r="A62" s="100" t="s">
         <v>43</v>
       </c>
       <c r="B62" s="46" t="s">
@@ -9642,7 +9650,7 @@
       </c>
     </row>
     <row r="63" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A63" s="94"/>
+      <c r="A63" s="100"/>
       <c r="B63" s="59" t="s">
         <v>53</v>
       </c>
@@ -9672,7 +9680,7 @@
       </c>
     </row>
     <row r="64" spans="1:14" s="20" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="94"/>
+      <c r="A64" s="100"/>
       <c r="B64" s="60" t="s">
         <v>54</v>
       </c>
@@ -9702,7 +9710,7 @@
       </c>
     </row>
     <row r="65" spans="1:11" s="20" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A65" s="94"/>
+      <c r="A65" s="100"/>
       <c r="B65" s="48" t="s">
         <v>46</v>
       </c>
@@ -9732,7 +9740,7 @@
       </c>
     </row>
     <row r="66" spans="1:11" s="20" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A66" s="94"/>
+      <c r="A66" s="100"/>
       <c r="B66" s="60" t="s">
         <v>56</v>
       </c>
@@ -9762,7 +9770,7 @@
       </c>
     </row>
     <row r="67" spans="1:11" s="20" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A67" s="94"/>
+      <c r="A67" s="100"/>
       <c r="B67" s="18" t="s">
         <v>48</v>
       </c>
@@ -9792,7 +9800,7 @@
       </c>
     </row>
     <row r="68" spans="1:11" s="20" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A68" s="94"/>
+      <c r="A68" s="100"/>
       <c r="B68" s="18" t="s">
         <v>57</v>
       </c>
@@ -10043,21 +10051,21 @@
     </row>
     <row r="91" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="92" spans="1:10" ht="28.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A92" s="95" t="s">
+      <c r="A92" s="105" t="s">
         <v>60</v>
       </c>
-      <c r="B92" s="96"/>
-      <c r="C92" s="96"/>
-      <c r="D92" s="96"/>
-      <c r="E92" s="96"/>
-      <c r="F92" s="96"/>
+      <c r="B92" s="95"/>
+      <c r="C92" s="95"/>
+      <c r="D92" s="95"/>
+      <c r="E92" s="95"/>
+      <c r="F92" s="95"/>
       <c r="G92" s="97"/>
       <c r="H92" s="98"/>
       <c r="I92" s="45"/>
       <c r="J92" s="45"/>
     </row>
     <row r="93" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A93" s="99" t="s">
+      <c r="A93" s="106" t="s">
         <v>43</v>
       </c>
       <c r="B93" s="46" t="s">
@@ -10077,7 +10085,7 @@
       </c>
     </row>
     <row r="94" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A94" s="100"/>
+      <c r="A94" s="107"/>
       <c r="B94" s="48" t="s">
         <v>45</v>
       </c>
@@ -10095,7 +10103,7 @@
       </c>
     </row>
     <row r="95" spans="1:10" s="20" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A95" s="100"/>
+      <c r="A95" s="107"/>
       <c r="B95" s="60" t="s">
         <v>46</v>
       </c>
@@ -10113,7 +10121,7 @@
       </c>
     </row>
     <row r="96" spans="1:10" s="20" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A96" s="100"/>
+      <c r="A96" s="107"/>
       <c r="B96" s="48" t="s">
         <v>48</v>
       </c>
@@ -10259,21 +10267,21 @@
     </row>
     <row r="113" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="114" spans="1:10" ht="28.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A114" s="101" t="s">
+      <c r="A114" s="94" t="s">
         <v>61</v>
       </c>
-      <c r="B114" s="96"/>
-      <c r="C114" s="96"/>
-      <c r="D114" s="96"/>
-      <c r="E114" s="96"/>
-      <c r="F114" s="96"/>
+      <c r="B114" s="95"/>
+      <c r="C114" s="95"/>
+      <c r="D114" s="95"/>
+      <c r="E114" s="95"/>
+      <c r="F114" s="95"/>
       <c r="G114" s="97"/>
       <c r="H114" s="98"/>
       <c r="I114" s="45"/>
       <c r="J114" s="45"/>
     </row>
     <row r="115" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A115" s="94" t="s">
+      <c r="A115" s="100" t="s">
         <v>43</v>
       </c>
       <c r="B115" s="46" t="s">
@@ -10293,7 +10301,7 @@
       </c>
     </row>
     <row r="116" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A116" s="94"/>
+      <c r="A116" s="100"/>
       <c r="B116" s="48" t="s">
         <v>45</v>
       </c>
@@ -10311,7 +10319,7 @@
       </c>
     </row>
     <row r="117" spans="1:10" s="20" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A117" s="94"/>
+      <c r="A117" s="100"/>
       <c r="B117" s="18" t="s">
         <v>46</v>
       </c>
@@ -10457,6 +10465,13 @@
     </row>
   </sheetData>
   <mergeCells count="14">
+    <mergeCell ref="A115:A117"/>
+    <mergeCell ref="A62:A68"/>
+    <mergeCell ref="A92:F92"/>
+    <mergeCell ref="G92:H92"/>
+    <mergeCell ref="A93:A96"/>
+    <mergeCell ref="A114:F114"/>
+    <mergeCell ref="G114:H114"/>
     <mergeCell ref="A61:J61"/>
     <mergeCell ref="K61:L61"/>
     <mergeCell ref="A1:J1"/>
@@ -10464,13 +10479,6 @@
     <mergeCell ref="A30:J30"/>
     <mergeCell ref="K30:L30"/>
     <mergeCell ref="A31:A39"/>
-    <mergeCell ref="A115:A117"/>
-    <mergeCell ref="A62:A68"/>
-    <mergeCell ref="A92:F92"/>
-    <mergeCell ref="G92:H92"/>
-    <mergeCell ref="A93:A96"/>
-    <mergeCell ref="A114:F114"/>
-    <mergeCell ref="G114:H114"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -10488,18 +10496,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="27" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="83" t="s">
+      <c r="A1" s="85" t="s">
         <v>62</v>
       </c>
-      <c r="B1" s="84"/>
-      <c r="C1" s="84"/>
-      <c r="D1" s="84"/>
-      <c r="E1" s="84"/>
-      <c r="F1" s="84"/>
-      <c r="G1" s="84"/>
-      <c r="H1" s="84"/>
-      <c r="I1" s="84"/>
-      <c r="J1" s="85"/>
+      <c r="B1" s="86"/>
+      <c r="C1" s="86"/>
+      <c r="D1" s="86"/>
+      <c r="E1" s="86"/>
+      <c r="F1" s="86"/>
+      <c r="G1" s="86"/>
+      <c r="H1" s="86"/>
+      <c r="I1" s="86"/>
+      <c r="J1" s="87"/>
     </row>
     <row r="2" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
@@ -10588,11 +10596,11 @@
     </row>
     <row r="10" spans="1:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="11" spans="1:11" ht="29.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="G11" s="92" t="s">
+      <c r="G11" s="83" t="s">
         <v>8</v>
       </c>
-      <c r="H11" s="93"/>
-      <c r="I11" s="93"/>
+      <c r="H11" s="84"/>
+      <c r="I11" s="84"/>
       <c r="J11" s="42">
         <f>J5</f>
         <v>146</v>
@@ -10628,14 +10636,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="28.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="95" t="s">
+      <c r="A1" s="105" t="s">
         <v>65</v>
       </c>
-      <c r="B1" s="96"/>
-      <c r="C1" s="96"/>
-      <c r="D1" s="96"/>
-      <c r="E1" s="96"/>
-      <c r="F1" s="96"/>
+      <c r="B1" s="95"/>
+      <c r="C1" s="95"/>
+      <c r="D1" s="95"/>
+      <c r="E1" s="95"/>
+      <c r="F1" s="95"/>
       <c r="G1" s="97" t="s">
         <v>42</v>
       </c>
@@ -10644,7 +10652,7 @@
       <c r="J1" s="45"/>
     </row>
     <row r="2" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="99" t="s">
+      <c r="A2" s="106" t="s">
         <v>43</v>
       </c>
       <c r="B2" s="46" t="s">
@@ -10664,7 +10672,7 @@
       </c>
     </row>
     <row r="3" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="100"/>
+      <c r="A3" s="107"/>
       <c r="B3" s="59" t="s">
         <v>53</v>
       </c>
@@ -10682,7 +10690,7 @@
       </c>
     </row>
     <row r="4" spans="1:10" s="20" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="100"/>
+      <c r="A4" s="107"/>
       <c r="B4" s="60" t="s">
         <v>54</v>
       </c>
@@ -10700,7 +10708,7 @@
       </c>
     </row>
     <row r="5" spans="1:10" s="20" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="100"/>
+      <c r="A5" s="107"/>
       <c r="B5" s="48" t="s">
         <v>66</v>
       </c>
@@ -10718,7 +10726,7 @@
       </c>
     </row>
     <row r="6" spans="1:10" s="20" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="100"/>
+      <c r="A6" s="107"/>
       <c r="B6" s="48" t="s">
         <v>46</v>
       </c>
@@ -10736,7 +10744,7 @@
       </c>
     </row>
     <row r="7" spans="1:10" s="20" customFormat="1" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="100"/>
+      <c r="A7" s="107"/>
       <c r="B7" s="61">
         <v>46052</v>
       </c>
@@ -10920,20 +10928,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="27" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="83" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="84"/>
-      <c r="C1" s="84"/>
-      <c r="D1" s="84"/>
-      <c r="E1" s="84"/>
-      <c r="F1" s="84"/>
-      <c r="G1" s="84"/>
-      <c r="H1" s="84"/>
-      <c r="I1" s="84"/>
-      <c r="J1" s="84"/>
-      <c r="K1" s="84"/>
-      <c r="L1" s="85"/>
+      <c r="A1" s="85" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="86"/>
+      <c r="C1" s="86"/>
+      <c r="D1" s="86"/>
+      <c r="E1" s="86"/>
+      <c r="F1" s="86"/>
+      <c r="G1" s="86"/>
+      <c r="H1" s="86"/>
+      <c r="I1" s="86"/>
+      <c r="J1" s="86"/>
+      <c r="K1" s="86"/>
+      <c r="L1" s="87"/>
     </row>
     <row r="2" spans="1:13" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
@@ -11628,18 +11636,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="27" customHeight="1" thickBot="1" x14ac:dyDescent="0.45">
-      <c r="A1" s="83" t="s">
+      <c r="A1" s="85" t="s">
         <v>68</v>
       </c>
-      <c r="B1" s="84"/>
-      <c r="C1" s="84"/>
-      <c r="D1" s="84"/>
-      <c r="E1" s="84"/>
-      <c r="F1" s="84"/>
-      <c r="G1" s="84"/>
-      <c r="H1" s="84"/>
-      <c r="I1" s="84"/>
-      <c r="J1" s="85"/>
+      <c r="B1" s="86"/>
+      <c r="C1" s="86"/>
+      <c r="D1" s="86"/>
+      <c r="E1" s="86"/>
+      <c r="F1" s="86"/>
+      <c r="G1" s="86"/>
+      <c r="H1" s="86"/>
+      <c r="I1" s="86"/>
+      <c r="J1" s="87"/>
     </row>
     <row r="2" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
@@ -11883,11 +11891,11 @@
     </row>
     <row r="18" spans="7:11" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="19" spans="7:11" ht="29.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="G19" s="92" t="s">
+      <c r="G19" s="83" t="s">
         <v>8</v>
       </c>
-      <c r="H19" s="93"/>
-      <c r="I19" s="93"/>
+      <c r="H19" s="84"/>
+      <c r="I19" s="84"/>
       <c r="J19" s="42">
         <f>J5+J10+J15</f>
         <v>150</v>

</xml_diff>